<commit_message>
session 20260904 (developer mode): #1444 catalogue-code-split migration + #1383 verse-lexical Window 1 Layer 1/Layer 2 full build (schema/config/code/PS, 552k-row backfill, 2 live bugs caught+fixed) -- both approved; #1383 leftovers spawned as #1448-1451, ps-tools worksheet fixed; #1447 glossary built full-scope (18 T1-T9 entries), 1446 range/deprecation error corrected, stale prose_section FK found+worked around (spawned #1452, build recorded as #1453); escalation-backlog check worked to real completion -- #1441 genuine data-integrity fix (824-verse FK-orphan repair), #1442 confirmed addressed, #1378/#1379 substantively reviewed and handed back
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -172,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -237,6 +237,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5097,7 +5101,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5105,6 +5109,7 @@
     <col width="22" bestFit="1" customWidth="1" min="3" max="7"/>
     <col width="11.42578125" bestFit="1" customWidth="1" min="8" max="8"/>
     <col width="13.5703125" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -5168,6 +5173,11 @@
           <t>-Step</t>
         </is>
       </c>
+      <c r="J4" s="23" t="inlineStr">
+        <is>
+          <t>-PayloadPath</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="51.75" customFormat="1" customHeight="1" s="18">
       <c r="D5" s="17" t="inlineStr">
@@ -5182,7 +5192,12 @@
       </c>
       <c r="I5" s="18" t="inlineStr">
         <is>
-          <t>lexical.build|report.verse_lexical -- omit to run both chained; report.verse_lexical alone VIEWS already-built results with no re-build</t>
+          <t>lexical.build|lexical.enrich|report.verse_lexical|report.lexical_exceptions|report.lexical_extract -- omit to run the full chained sequence (now also runs lexical.enrich + report.lexical_exceptions); report.verse_lexical alone VIEWS already-built results with no re-build</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>path to the lexical.enrich payload JSON (notes/remove/genre) -- REQUIRED when -Step lexical.enrich is used, or when running the full sequence (which now includes lexical.enrich)</t>
         </is>
       </c>
     </row>
@@ -5193,7 +5208,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")</f>
         <v/>
       </c>
       <c r="C6" s="18" t="inlineStr">
@@ -5721,12 +5736,14 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="22" bestFit="1" customWidth="1" min="3" max="7"/>
+    <col width="11.4" customWidth="1" min="8" max="8"/>
+    <col width="11.4" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -5780,6 +5797,16 @@
           <t>-Trace</t>
         </is>
       </c>
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>-Suggest</t>
+        </is>
+      </c>
+      <c r="I4" s="22" t="inlineStr">
+        <is>
+          <t>-Confirm</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="F5" s="17" t="inlineStr">
@@ -5787,6 +5814,16 @@
           <t>path to the payload JSON</t>
         </is>
       </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>switch -- propose the next candidate passage boundary from cheap mechanical proxy signals (no table write, pauses for confirm/adjust); mutually exclusive with -Chapters/-Range</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>switch -- only with -Suggest: accept the suggestion verbatim, straight into passage.build (still needs -PayloadPath)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
@@ -5795,7 +5832,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")&amp;IF(I6&lt;&gt;"",$I$4&amp;" ","")</f>
         <v/>
       </c>
     </row>

</xml_diff>